<commit_message>
Update BNP Paribas Open projections
</commit_message>
<xml_diff>
--- a/draws/iw2026.xlsx
+++ b/draws/iw2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cadecarlson/EDACCloud/Development/tf-site/draws/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{200116B0-C698-7040-9690-9ED0D8D2DDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9289F61-3B78-3B42-BADA-3682F4B2DBA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -791,7 +791,7 @@
         <v>18</v>
       </c>
       <c r="D2" s="2">
-        <v>2270</v>
+        <v>2240</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
@@ -2569,7 +2569,7 @@
         <v>110</v>
       </c>
       <c r="D129" s="2">
-        <v>2235</v>
+        <v>2210</v>
       </c>
       <c r="E129" s="2">
         <v>1</v>

</xml_diff>